<commit_message>
Gera e processa segunda execucao
</commit_message>
<xml_diff>
--- a/Projeto/resultados_testes_estatisticos_v1.xlsx
+++ b/Projeto/resultados_testes_estatisticos_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gilcesarf/git/repositories/imd/imd3002-202502/Projeto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83695C16-2D2E-8142-98A5-35B32D082FCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00EE9C9C-3758-5A46-90AF-7DDBF8943697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37080" yWindow="3240" windowWidth="34560" windowHeight="12940" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36200" yWindow="1540" windowWidth="34560" windowHeight="9840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumo_Geral" sheetId="1" r:id="rId1"/>
@@ -150,9 +150,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="_-* #,##0.000000_-;\-* #,##0.000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="172" formatCode="_-* #,##0.000000000_-;\-* #,##0.000000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.000000_-;\-* #,##0.000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.000000000_-;\-* #,##0.000000000_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -193,9 +193,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -571,7 +571,7 @@
       <c r="D2">
         <v>7.209326424870441</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="3">
         <v>0.6153355838888005</v>
       </c>
       <c r="F2" t="s">
@@ -612,7 +612,7 @@
       <c r="D3">
         <v>4.8025980641874577</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="3">
         <v>0.85116553652812443</v>
       </c>
       <c r="F3" t="s">
@@ -653,7 +653,7 @@
       <c r="D4">
         <v>24.150537634408579</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="3">
         <v>5.698720869286655E-6</v>
       </c>
       <c r="F4" t="s">
@@ -694,7 +694,7 @@
       <c r="D5">
         <v>32.069331983805661</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="3">
         <v>1.9370733297032321E-4</v>
       </c>
       <c r="F5" t="s">

</xml_diff>